<commit_message>
Neutral axis labels on the maps and numeric order of trap identifiers
Axis titles no longer carry a hemisphere letter next to signed decimal degrees, and the High-High trap lists in the tables are ordered numerically (N°7 before N°10). Outputs regenerated; no statistic changed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tables.xlsx
+++ b/output/tables.xlsx
@@ -22131,7 +22131,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>N°44, N°7</t>
+          <t>N°7, N°44</t>
         </is>
       </c>
     </row>
@@ -22173,7 +22173,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>N°12, N°45, N°51, N°63, N°65, N°69, N°7, N°79, N°82</t>
+          <t>N°7, N°12, N°45, N°51, N°63, N°65, N°69, N°79, N°82</t>
         </is>
       </c>
     </row>
@@ -22257,7 +22257,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>N°61, N°62, N°65, N°7, N°92</t>
+          <t>N°7, N°61, N°62, N°65, N°92</t>
         </is>
       </c>
     </row>
@@ -22299,7 +22299,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>N°106, N°108, N°127, N°128, N°136, N°49, N°52, N°55</t>
+          <t>N°49, N°52, N°55, N°106, N°108, N°127, N°128, N°136</t>
         </is>
       </c>
     </row>
@@ -22341,7 +22341,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>N°10, N°45, N°63, N°64, N°7, N°9</t>
+          <t>N°7, N°9, N°10, N°45, N°63, N°64</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renumber the supplementary tables and figures in the order of first citation in the manuscript
Sheet names S2 (Moran's I by k), S4 (class distribution), S5 (Kruskal-Wallis by scenario) and S6-S9 (Dunn tests), and figure files S1 (seasonal LISA maps), S2 (hotspot stability) and S3 (leave-one-event-out validation), now match the revised manuscript. No statistic changed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tables.xlsx
+++ b/output/tables.xlsx
@@ -11,17 +11,17 @@
     <sheet name="trap_activity" sheetId="2" r:id="rId2"/>
     <sheet name="traps_per_season" sheetId="3" r:id="rId3"/>
     <sheet name="moran_by_season" sheetId="4" r:id="rId4"/>
-    <sheet name="S1_moran_by_k" sheetId="5" r:id="rId5"/>
+    <sheet name="S2_moran_by_k" sheetId="5" r:id="rId5"/>
     <sheet name="cluster_geometry" sheetId="6" r:id="rId6"/>
     <sheet name="moran_common_sets" sheetId="7" r:id="rId7"/>
     <sheet name="lisa_by_season" sheetId="8" r:id="rId8"/>
     <sheet name="class_summary" sheetId="9" r:id="rId9"/>
-    <sheet name="S2_class_distribution" sheetId="10" r:id="rId10"/>
-    <sheet name="S3_kruskal_by_scenario" sheetId="11" r:id="rId11"/>
-    <sheet name="S4_dunn_S1_and_S4" sheetId="12" r:id="rId12"/>
-    <sheet name="S5_dunn_S2" sheetId="13" r:id="rId13"/>
-    <sheet name="S6_dunn_S3" sheetId="14" r:id="rId14"/>
-    <sheet name="S7_dunn_S5" sheetId="15" r:id="rId15"/>
+    <sheet name="S4_class_distribution" sheetId="10" r:id="rId10"/>
+    <sheet name="S5_kruskal_by_scenario" sheetId="11" r:id="rId11"/>
+    <sheet name="S6_dunn_S1_and_S4" sheetId="12" r:id="rId12"/>
+    <sheet name="S7_dunn_S2" sheetId="13" r:id="rId13"/>
+    <sheet name="S8_dunn_S3" sheetId="14" r:id="rId14"/>
+    <sheet name="S9_dunn_S5" sheetId="15" r:id="rId15"/>
     <sheet name="critical_events" sheetId="16" r:id="rId16"/>
     <sheet name="insecticide_applications" sheetId="17" r:id="rId17"/>
     <sheet name="moran_global" sheetId="18" r:id="rId18"/>

</xml_diff>